<commit_message>
updated the sample data to reflect the changes in the jupyter notebook
</commit_message>
<xml_diff>
--- a/sample_data/in_test_data/rhodo_test_data.xlsx
+++ b/sample_data/in_test_data/rhodo_test_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10811"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mahl006/git_repos/valpas-prototype/sample_data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mahl006/git_repos/valpas-prototype/sample_data/in_test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{34980960-2060-364A-B0C5-C3C29BE96D3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C5B15F9-C2E2-9447-AA73-01D3F1B0C226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="24780" yWindow="7500" windowWidth="27640" windowHeight="16940" xr2:uid="{3AEE8229-5F5B-1643-9AE0-C8D66700B705}"/>
   </bookViews>

</xml_diff>

<commit_message>
updated sample data for testing
</commit_message>
<xml_diff>
--- a/sample_data/in_test_data/rhodo_test_data.xlsx
+++ b/sample_data/in_test_data/rhodo_test_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10916"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11110"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/mahl006/git_repos/valpas-prototype/sample_data/in_test_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C5B15F9-C2E2-9447-AA73-01D3F1B0C226}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B675C4B6-BFFD-AA4B-A33B-CAE24BF528AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="24780" yWindow="7500" windowWidth="27640" windowHeight="16940" xr2:uid="{3AEE8229-5F5B-1643-9AE0-C8D66700B705}"/>
+    <workbookView xWindow="36220" yWindow="12180" windowWidth="27640" windowHeight="16940" xr2:uid="{3AEE8229-5F5B-1643-9AE0-C8D66700B705}"/>
   </bookViews>
   <sheets>
     <sheet name="Proteomics" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="13">
   <si>
     <t>Metabolite</t>
   </si>
@@ -49,9 +49,6 @@
   </si>
   <si>
     <t>X_SD_exp</t>
-  </si>
-  <si>
-    <t>X_SD_stat</t>
   </si>
   <si>
     <t>A_SD_exp</t>
@@ -455,7 +452,7 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B1" t="s">
         <v>1</v>
@@ -467,10 +464,10 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
         <v>5</v>
-      </c>
-      <c r="F1" t="s">
-        <v>6</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
@@ -580,10 +577,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF7ACEDD-D7E7-CA4C-A499-2A3F6A02C679}">
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -605,24 +602,21 @@
       <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
+      <c r="F2">
+        <v>128</v>
+      </c>
+      <c r="G2">
+        <v>2975</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
         <v>8</v>
-      </c>
-      <c r="G2">
-        <v>128</v>
-      </c>
-      <c r="H2">
-        <v>2975</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A3" t="s">
-        <v>9</v>
       </c>
       <c r="B3">
         <v>725</v>
@@ -634,18 +628,15 @@
         <v>844</v>
       </c>
       <c r="E3">
-        <v>450</v>
+        <v>1312</v>
       </c>
       <c r="F3">
-        <v>1312</v>
-      </c>
-      <c r="G3">
         <v>5178</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B4">
         <v>3</v>
@@ -657,41 +648,35 @@
         <v>3348</v>
       </c>
       <c r="E4">
-        <v>319</v>
+        <v>4</v>
       </c>
       <c r="F4">
-        <v>4</v>
-      </c>
-      <c r="G4">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5">
+        <v>0</v>
+      </c>
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
+        <v>588</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
         <v>11</v>
-      </c>
-      <c r="B5">
-        <v>0</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>0</v>
-      </c>
-      <c r="E5">
-        <v>0</v>
-      </c>
-      <c r="F5">
-        <v>0</v>
-      </c>
-      <c r="G5">
-        <v>588</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A6" t="s">
-        <v>12</v>
       </c>
       <c r="B6">
         <v>1263</v>
@@ -703,12 +688,9 @@
         <v>518</v>
       </c>
       <c r="E6">
-        <v>155</v>
+        <v>1741</v>
       </c>
       <c r="F6">
-        <v>1741</v>
-      </c>
-      <c r="G6">
         <v>1748</v>
       </c>
     </row>

</xml_diff>